<commit_message>
Update property registration and workbook
</commit_message>
<xml_diff>
--- a/2026年度物件表_KMN置換_列移動_2026-10-10.xlsx
+++ b/2026年度物件表_KMN置換_列移動_2026-10-10.xlsx
@@ -11640,64 +11640,54 @@
       <c r="AC117" s="210"/>
     </row>
     <row r="118" spans="1:29" s="213" customFormat="1" ht="21" customHeight="1">
-      <c r="A118" s="241" t="s">
-        <v>245</v>
-      </c>
-      <c r="B118" s="206" t="s">
-        <v>24</v>
+      <c r="A118" s="241" t="inlineStr">
+        <is>
+          <t>白鳳通り</t>
+        </is>
+      </c>
+      <c r="B118" s="206" t="inlineStr">
+        <is>
+          <t xml:space="preserve">会社　商店</t>
+        </is>
       </c>
       <c r="C118" s="242">
         <v>117</v>
       </c>
       <c r="D118" s="206">
-        <v>116</v>
-      </c>
-      <c r="E118" s="206" t="s">
-        <v>258</v>
+        <v>291</v>
+      </c>
+      <c r="E118" s="206" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ビークイック　ジム</t>
+        </is>
       </c>
       <c r="F118" s="206"/>
-      <c r="G118" s="206" t="s">
-        <v>259</v>
-      </c>
-      <c r="H118" s="206" t="s">
-        <v>27</v>
-      </c>
-      <c r="I118" s="206" t="s">
-        <v>27</v>
-      </c>
-      <c r="J118" s="206" t="s">
-        <v>27</v>
-      </c>
-      <c r="K118" s="216" t="s">
-        <v>27</v>
-      </c>
-      <c r="L118" s="206" t="s">
-        <v>27</v>
+      <c r="H118" s="206"/>
+      <c r="I118" s="206" t="inlineStr">
+        <is>
+          <t>N-</t>
+        </is>
+      </c>
+      <c r="J118" s="206"/>
+      <c r="K118" s="216"/>
+      <c r="L118" s="206" t="inlineStr">
+        <is>
+          <t>N-</t>
+        </is>
       </c>
       <c r="M118" s="206"/>
-      <c r="N118" s="206"/>
-      <c r="O118" s="206" t="s">
-        <v>13</v>
-      </c>
       <c r="P118" s="206"/>
-      <c r="Q118" s="206"/>
-      <c r="R118" s="217"/>
-      <c r="S118" s="206"/>
-      <c r="T118" s="218"/>
-      <c r="U118" s="206" t="s">
-        <v>37</v>
-      </c>
-      <c r="V118" s="206" t="s">
-        <v>29</v>
-      </c>
-      <c r="W118" s="206" t="s">
-        <v>43</v>
-      </c>
-      <c r="X118" s="206" t="s">
-        <v>38</v>
-      </c>
-      <c r="Y118" s="206" t="s">
-        <v>30</v>
+      <c r="V118" s="206" t="inlineStr">
+        <is>
+          <t>㊋</t>
+        </is>
+      </c>
+      <c r="W118" s="206"/>
+      <c r="X118" s="206"/>
+      <c r="Y118" s="206" t="inlineStr">
+        <is>
+          <t>㊎</t>
+        </is>
       </c>
       <c r="Z118" s="206"/>
       <c r="AA118" s="208"/>

</xml_diff>